<commit_message>
Recalculate team costs with updated wages
Usta 120k, çırak 60k, mühendis 70k brüt/ay; refresh expense and
profit tables for kırık 450 scenario.

Co-authored-by: barsokrr <barsokrr@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/metraj/Ekip_Gider_Kirilimi.xlsx
+++ b/metraj/Ekip_Gider_Kirilimi.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="EKIP GIDER" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="OZET" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -41,6 +42,11 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="13"/>
     </font>
   </fonts>
   <fills count="5">
@@ -84,7 +90,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -98,8 +104,12 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -465,41 +475,41 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H31"/>
+  <dimension ref="A1:H32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
     <col width="28" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>EKİP GİDER KIRILIMI — NASIL HESAPLANDI?</t>
+          <t>EKİP GİDER KIRILIMI — GÜNCEL MAAŞLAR</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Senaryo: 2 usta + 3 çırak + 1 mühendis (4A) + şirket sahibi (4B) | Süre: 6 ay | Kırık 450 işi</t>
+          <t>Usta 120.000 · Çırak 60.000 · Mühendis 70.000 TL/ay brüt | 2+3+1 | 6 ay | Kırık 450</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>A) PERSONEL ÜCRETLERİ (brüt varsayım)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="32" customHeight="1">
+          <t>A) PERSONEL ÜCRETLERİ</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Kalem</t>
@@ -512,12 +522,12 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Brüt / kişi / ay (TL)</t>
+          <t>Brüt / kişi / ay</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Aylık toplam (TL)</t>
+          <t>Aylık toplam</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -527,12 +537,12 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Dönem toplam (TL)</t>
+          <t>Dönem toplam</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>Hesap formülü</t>
+          <t>Formül</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
@@ -551,20 +561,20 @@
         <v>2</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>55000</v>
+        <v>120000</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>110000</v>
+        <v>240000</v>
       </c>
       <c r="E6" s="4" t="n">
         <v>6</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>660000</v>
+        <v>1440000</v>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>2 × 55.000 × 6</t>
+          <t>2 × 120.000 × 6</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
@@ -583,20 +593,20 @@
         <v>3</v>
       </c>
       <c r="C7" s="5" t="n">
-        <v>28000</v>
+        <v>60000</v>
       </c>
       <c r="D7" s="5" t="n">
-        <v>84000</v>
+        <v>180000</v>
       </c>
       <c r="E7" s="4" t="n">
         <v>6</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>504000</v>
+        <v>1080000</v>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>3 × 28.000 × 6</t>
+          <t>3 × 60.000 × 6</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
@@ -615,20 +625,20 @@
         <v>1</v>
       </c>
       <c r="C8" s="5" t="n">
-        <v>65000</v>
+        <v>70000</v>
       </c>
       <c r="D8" s="5" t="n">
-        <v>65000</v>
+        <v>70000</v>
       </c>
       <c r="E8" s="4" t="n">
         <v>6</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>390000</v>
+        <v>420000</v>
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>1 × 65.000 × 6</t>
+          <t>1 × 70.000 × 6</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
@@ -646,15 +656,15 @@
       <c r="B9" s="6" t="n"/>
       <c r="C9" s="6" t="n"/>
       <c r="D9" s="7" t="n">
-        <v>259000</v>
+        <v>490000</v>
       </c>
       <c r="E9" s="6" t="n"/>
       <c r="F9" s="7" t="n">
-        <v>1554000</v>
+        <v>2940000</v>
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>660.000 + 504.000 + 390.000</t>
+          <t>1440000 + 1080000 + 420000</t>
         </is>
       </c>
       <c r="H9" s="6" t="n"/>
@@ -662,7 +672,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>B) ÜCRET DIŞI GİDERLER</t>
+          <t>B) ÜCRET DIŞI</t>
         </is>
       </c>
     </row>
@@ -684,7 +694,7 @@
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>Dönem tutar (TL)</t>
+          <t>Dönem tutar</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr">
@@ -696,7 +706,7 @@
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>İşveren SGK + işsizlik</t>
+          <t>İşveren SGK ~%22,5</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
@@ -706,22 +716,22 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>1.554.000 × 0.225</t>
+          <t>2.940.000 × 0.225</t>
         </is>
       </c>
       <c r="D13" s="5" t="n">
-        <v>349650</v>
+        <v>661500</v>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Kabaca; teşvik MM ile netleşir</t>
+          <t>Kabaca</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>Bağ-Kur (şirket sahibi)</t>
+          <t>Bağ-Kur (sahip)</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
@@ -731,7 +741,7 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>10000 × 6</t>
+          <t>10000×6</t>
         </is>
       </c>
       <c r="D14" s="5" t="n">
@@ -739,7 +749,7 @@
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>Sahip maaşlı değil</t>
+          <t>Maaş yok</t>
         </is>
       </c>
     </row>
@@ -756,22 +766,18 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>5000 × 6</t>
+          <t>5000×6</t>
         </is>
       </c>
       <c r="D15" s="5" t="n">
         <v>30000</v>
       </c>
-      <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t>Beyanname + defter</t>
-        </is>
-      </c>
+      <c r="E15" s="4" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>İSG / eğitim / MYB</t>
+          <t>İSG / MYB</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
@@ -781,22 +787,18 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>dönem sabit</t>
+          <t>dönem</t>
         </is>
       </c>
       <c r="D16" s="5" t="n">
         <v>80000</v>
       </c>
-      <c r="E16" s="4" t="inlineStr">
-        <is>
-          <t>Çok tehlikeli sınıf</t>
-        </is>
-      </c>
+      <c r="E16" s="4" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>Küçük sarf</t>
+          <t>Sarf</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
@@ -806,7 +808,7 @@
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>dönem sabit</t>
+          <t>dönem</t>
         </is>
       </c>
       <c r="D17" s="5" t="n">
@@ -814,14 +816,14 @@
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>Kalıp malzemesi hariç</t>
+          <t>Malzeme hariç</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>Ulaşım / iletişim / diğer</t>
+          <t>Diğer</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
@@ -831,7 +833,7 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>dönem sabit</t>
+          <t>dönem</t>
         </is>
       </c>
       <c r="D18" s="5" t="n">
@@ -848,18 +850,14 @@
       <c r="B19" s="10" t="n"/>
       <c r="C19" s="10" t="n"/>
       <c r="D19" s="11" t="n">
-        <v>2253650</v>
-      </c>
-      <c r="E19" s="10" t="inlineStr">
-        <is>
-          <t>Ücret + SGK + Bağ-Kur + muhasebe + İSG + sarf + diğer</t>
-        </is>
-      </c>
+        <v>3951500</v>
+      </c>
+      <c r="E19" s="10" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>C) KÂRA BAĞLANTI (hatırlatma)</t>
+          <t>C) KÂR</t>
         </is>
       </c>
     </row>
@@ -880,7 +878,7 @@
         </is>
       </c>
       <c r="B23" s="12" t="n">
-        <v>2253650</v>
+        <v>3951500</v>
       </c>
     </row>
     <row r="24">
@@ -890,68 +888,209 @@
         </is>
       </c>
       <c r="B24" s="12" t="n">
-        <v>3044380</v>
+        <v>1346530</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Tahmini net kâr (GV sonrası kabaca)</t>
+          <t>Tahmini GV (dilimli kabaca)</t>
         </is>
       </c>
       <c r="B25" s="12" t="n">
-        <v>2032628</v>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Dilimler varsayımsal</t>
-        </is>
+        <v>403285.5</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Damga / beyanname</t>
+        </is>
+      </c>
+      <c r="B26" s="12" t="n">
+        <v>12000</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>NOTLAR</t>
-        </is>
+      <c r="A27" s="13" t="inlineStr">
+        <is>
+          <t>NET KÂR (GV sonrası)</t>
+        </is>
+      </c>
+      <c r="B27" s="14" t="n">
+        <v>931244.5</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>1) Brüt ücretler piyasa varsayımıdır; bordro net/brüt farkı MM ile kesinleşir.</t>
-        </is>
+          <t>Sahip çekimi 40k×6 (opsiyonel)</t>
+        </is>
+      </c>
+      <c r="B28" s="12" t="n">
+        <v>240000</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2) SGK %22,5 kabaca işveren payıdır (teşvik/indirim hariç).</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>3) Şirket sahibi için maaş yazılmaz; Bağ-Kur prim + isteğe bağlı kârdan çekim vardır (çekim bu tablonun işletme giderine dahil değildir).</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>4) Kalıp malzemesi ve iskele müteahhitte varsayıldığı için giderde yoktur.</t>
+          <t>Çekim sonrası kalan</t>
+        </is>
+      </c>
+      <c r="B29" s="12" t="n">
+        <v>691244.5</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>NOT: Brüt ücret kullanıcı girdileridir. SGK/GV kesin hesabı mali müşavirindir. Sahip maaşı yoktur.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="A30:H30"/>
-    <mergeCell ref="A29:H29"/>
+  <mergeCells count="3">
+    <mergeCell ref="A32:H32"/>
     <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A28:H28"/>
     <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A31:H31"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="15" t="inlineStr">
+        <is>
+          <t>KISA ÖZET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="16" t="inlineStr">
+        <is>
+          <t>Kalem</t>
+        </is>
+      </c>
+      <c r="B3" s="16" t="inlineStr">
+        <is>
+          <t>Tutar TL</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2 usta × 120.000 × 6</t>
+        </is>
+      </c>
+      <c r="B4" s="12" t="n">
+        <v>1440000</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>3 çırak × 60.000 × 6</t>
+        </is>
+      </c>
+      <c r="B5" s="12" t="n">
+        <v>1080000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>1 mühendis × 70.000 × 6</t>
+        </is>
+      </c>
+      <c r="B6" s="12" t="n">
+        <v>420000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>4A ücret toplam</t>
+        </is>
+      </c>
+      <c r="B7" s="12" t="n">
+        <v>2940000</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>SGK %22,5</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="n">
+        <v>661500</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Bağ-Kur+muhasebe+İSG+sarf+diğer</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="n">
+        <v>350000</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="13" t="inlineStr">
+        <is>
+          <t>TOPLAM GİDER</t>
+        </is>
+      </c>
+      <c r="B10" s="14" t="n">
+        <v>3951500</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Matrah</t>
+        </is>
+      </c>
+      <c r="B11" s="12" t="n">
+        <v>5298030</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Vergi öncesi kâr</t>
+        </is>
+      </c>
+      <c r="B12" s="12" t="n">
+        <v>1346530</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t>NET KÂR (kabaca)</t>
+        </is>
+      </c>
+      <c r="B13" s="14" t="n">
+        <v>931244.5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>